<commit_message>
generador de ordenes de entrada en base a un formulario llenado en vue
</commit_message>
<xml_diff>
--- a/src/plantillas/entrada_plantilla.xlsx
+++ b/src/plantillas/entrada_plantilla.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\OneDrive\Desktop\inventario\inventoryHRAEI-back\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\OneDrive\Desktop\inventario\inventoryHRAEI-front\src\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89189458-45A8-4EF4-8286-AE666E7BA5FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5085D778-78DC-46D6-B35B-D965055F8E24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B2B4D7B8-25C3-42F1-81B4-952D6AD71DB5}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="90">
   <si>
     <t>NOMBRE DE INGENIERO RESIDENTE DE APOYO</t>
   </si>
@@ -301,6 +301,15 @@
   </si>
   <si>
     <t>{{descripcion.equip.entrada}}</t>
+  </si>
+  <si>
+    <t>{{observaciones.entrada}}</t>
+  </si>
+  <si>
+    <t>{{ing.apoyo.entrada}}</t>
+  </si>
+  <si>
+    <t>{{img.observaciones.entrada}}</t>
   </si>
 </sst>
 </file>
@@ -551,7 +560,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -686,10 +695,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -704,6 +709,18 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2826,10 +2843,10 @@
       <c r="A14" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="40" t="s">
+      <c r="B14" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="41"/>
+      <c r="C14" s="40"/>
       <c r="D14" s="34"/>
       <c r="E14" s="35"/>
       <c r="F14" s="35"/>
@@ -2839,8 +2856,8 @@
     </row>
     <row r="15" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="7"/>
-      <c r="B15" s="42"/>
-      <c r="C15" s="42"/>
+      <c r="B15" s="41"/>
+      <c r="C15" s="41"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
@@ -2849,17 +2866,17 @@
       <c r="I15" s="7"/>
     </row>
     <row r="16" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="43" t="s">
+      <c r="A16" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="43"/>
-      <c r="C16" s="43"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="43"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="43"/>
-      <c r="I16" s="43"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="42"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="42"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="42"/>
     </row>
     <row r="17" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
@@ -2950,17 +2967,17 @@
     </row>
     <row r="20" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="21" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="43"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-      <c r="H21" s="43"/>
-      <c r="I21" s="43"/>
+      <c r="B21" s="42"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="42"/>
+      <c r="I21" s="42"/>
     </row>
     <row r="22" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
@@ -3051,17 +3068,17 @@
     </row>
     <row r="25" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="43" t="s">
+      <c r="A26" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="43"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="43"/>
-      <c r="I26" s="43"/>
+      <c r="B26" s="42"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="42"/>
+      <c r="F26" s="42"/>
+      <c r="G26" s="42"/>
+      <c r="H26" s="42"/>
+      <c r="I26" s="42"/>
     </row>
     <row r="27" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
@@ -3152,17 +3169,17 @@
     </row>
     <row r="30" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="31" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="43" t="s">
+      <c r="A31" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="B31" s="43"/>
-      <c r="C31" s="43"/>
-      <c r="D31" s="43"/>
-      <c r="E31" s="43"/>
-      <c r="F31" s="43"/>
-      <c r="G31" s="43"/>
-      <c r="H31" s="43"/>
-      <c r="I31" s="43"/>
+      <c r="B31" s="42"/>
+      <c r="C31" s="42"/>
+      <c r="D31" s="42"/>
+      <c r="E31" s="42"/>
+      <c r="F31" s="42"/>
+      <c r="G31" s="42"/>
+      <c r="H31" s="42"/>
+      <c r="I31" s="42"/>
     </row>
     <row r="32" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
@@ -3237,15 +3254,19 @@
       <c r="I35" s="38"/>
     </row>
     <row r="36" spans="1:9" s="2" customFormat="1" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="39"/>
-      <c r="B36" s="39"/>
-      <c r="C36" s="39"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="39"/>
-      <c r="G36" s="39"/>
-      <c r="H36" s="39"/>
-      <c r="I36" s="39"/>
+      <c r="A36" s="43" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="44"/>
+      <c r="C36" s="44"/>
+      <c r="D36" s="44"/>
+      <c r="E36" s="45"/>
+      <c r="F36" s="43" t="s">
+        <v>89</v>
+      </c>
+      <c r="G36" s="44"/>
+      <c r="H36" s="44"/>
+      <c r="I36" s="45"/>
     </row>
     <row r="37" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="27" t="s">
@@ -3253,12 +3274,14 @@
       </c>
       <c r="B37" s="27"/>
       <c r="C37" s="27"/>
-      <c r="D37" s="40"/>
-      <c r="E37" s="40"/>
-      <c r="F37" s="40"/>
-      <c r="G37" s="40"/>
-      <c r="H37" s="40"/>
-      <c r="I37" s="40"/>
+      <c r="D37" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="39"/>
+      <c r="I37" s="39"/>
     </row>
     <row r="38" spans="1:9" s="2" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -3287,9 +3310,8 @@
     <row r="62" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="A35:I35"/>
-    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="D37:I37"/>
     <mergeCell ref="B14:C14"/>
@@ -3298,6 +3320,8 @@
     <mergeCell ref="A21:I21"/>
     <mergeCell ref="A26:I26"/>
     <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="F36:I36"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="A6:C6"/>

</xml_diff>